<commit_message>
reducing clutter in UI for operators
</commit_message>
<xml_diff>
--- a/ML Algorithm/data/_processed/Y labels/centrifuge_vacp_workload.xlsx
+++ b/ML Algorithm/data/_processed/Y labels/centrifuge_vacp_workload.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operators" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legend &amp; VACP Reference" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Step Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operators" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; VACP Reference" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operators'!$A$1:$K$290</definedName>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -114,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +161,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1554,11 +1558,11 @@
         </is>
       </c>
       <c r="I22" s="13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Discrete actuation (P2) [assumption]</t>
+          <t>Manipulation (P4) — release reclassified to background motor</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr"/>
@@ -1779,11 +1783,11 @@
         </is>
       </c>
       <c r="I27" s="13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>Discrete actuation (P2) [assumption]</t>
+          <t>Manipulation (P4) — release reclassified to background motor</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr"/>
@@ -3568,11 +3572,11 @@
         </is>
       </c>
       <c r="I66" s="13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Discrete actuation (P2) [assumption]</t>
+          <t>Manipulation (P4) — release reclassified to background motor</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr"/>
@@ -4858,11 +4862,11 @@
         </is>
       </c>
       <c r="I94" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J94" s="7" t="inlineStr">
         <is>
-          <t>Automatic (C1)</t>
+          <t>No cognitive activity (C0)</t>
         </is>
       </c>
       <c r="K94" s="7" t="inlineStr">
@@ -8322,11 +8326,11 @@
         </is>
       </c>
       <c r="I170" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J170" s="7" t="inlineStr">
         <is>
-          <t>Automatic (C1)</t>
+          <t>No cognitive activity (C0)</t>
         </is>
       </c>
       <c r="K170" s="7" t="inlineStr">
@@ -12064,11 +12068,11 @@
         </is>
       </c>
       <c r="I252" s="13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="J252" s="3" t="inlineStr">
         <is>
-          <t>Discrete actuation (P2) [assumption]</t>
+          <t>Manipulation (P4) — release reclassified to background motor</t>
         </is>
       </c>
       <c r="K252" s="3" t="inlineStr"/>
@@ -13430,11 +13434,11 @@
         </is>
       </c>
       <c r="I282" s="13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="J282" s="3" t="inlineStr">
         <is>
-          <t>Discrete actuation (P2) [assumption]</t>
+          <t>Manipulation (P4) — release reclassified to background motor</t>
         </is>
       </c>
       <c r="K282" s="3" t="inlineStr"/>
@@ -14093,39 +14097,48 @@
   </sheetPr>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Procedure</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Step ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Step description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Operators</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>MWI_step</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>MWI_max_recorded</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>p_normalized</t>
         </is>
@@ -14152,10 +14165,10 @@
         <v>23.8</v>
       </c>
       <c r="F2" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G2" t="n">
-        <v>0.137176</v>
+        <v>0.139753</v>
       </c>
     </row>
     <row r="3">
@@ -14176,13 +14189,13 @@
         <v>34</v>
       </c>
       <c r="E3" t="n">
-        <v>81</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G3" t="n">
-        <v>0.466859</v>
+        <v>0.449794</v>
       </c>
     </row>
     <row r="4">
@@ -14203,10 +14216,10 @@
         <v>102</v>
       </c>
       <c r="E4" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="F4" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -14230,13 +14243,13 @@
         <v>76</v>
       </c>
       <c r="E5" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F5" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G5" t="n">
-        <v>0.743516</v>
+        <v>0.751615</v>
       </c>
     </row>
     <row r="6">
@@ -14260,10 +14273,10 @@
         <v>25.6</v>
       </c>
       <c r="F6" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G6" t="n">
-        <v>0.14755</v>
+        <v>0.150323</v>
       </c>
     </row>
     <row r="7">
@@ -14284,13 +14297,13 @@
         <v>11</v>
       </c>
       <c r="E7" t="n">
-        <v>34.3</v>
+        <v>32.1</v>
       </c>
       <c r="F7" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G7" t="n">
-        <v>0.197695</v>
+        <v>0.188491</v>
       </c>
     </row>
     <row r="8">
@@ -14314,10 +14327,10 @@
         <v>64.40000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G8" t="n">
-        <v>0.371182</v>
+        <v>0.378156</v>
       </c>
     </row>
     <row r="9">
@@ -14338,13 +14351,13 @@
         <v>12</v>
       </c>
       <c r="E9" t="n">
-        <v>25.6</v>
+        <v>23.4</v>
       </c>
       <c r="F9" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G9" t="n">
-        <v>0.14755</v>
+        <v>0.137405</v>
       </c>
     </row>
     <row r="10">
@@ -14368,10 +14381,10 @@
         <v>13.9</v>
       </c>
       <c r="F10" t="n">
-        <v>173.5</v>
+        <v>170.3</v>
       </c>
       <c r="G10" t="n">
-        <v>0.08011500000000001</v>
+        <v>0.081621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>